<commit_message>
Anadir comparativa simulada 300 vs 1000 y actualizar Entregable 1
- scripts/comparativa_300_vs_1000.py + comparativa_300_vs_1000.xlsx:
  comparativa simulada 300 vs 1000 (motor reutilizado y validado contra la app).
- situacion_actual_300.xlsx + scripts/entregables_300_500.py: Entregable 1
  pasa a una unica columna de superficie (activada = min(derechos, ABRS)),
  sin SUPERFICIE_TOTAL_DESPUES_CAP.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/situacion_actual_300.xlsx
+++ b/situacion_actual_300.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -429,25 +429,20 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Superficie total declarada (ha)</t>
+          <t>Superficie activada (ha)</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Superficie con derecho / activada (ha)</t>
+          <t>Importe total (€)</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Importe total (€)</t>
+          <t>Nº de derechos</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
-        <is>
-          <t>Nº de derechos</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
         <is>
           <t>Importe medio (€/benef.)</t>
         </is>
@@ -463,18 +458,15 @@
         <v>1541</v>
       </c>
       <c r="C2" t="n">
-        <v>168296.15</v>
+        <v>87830.17999999999</v>
       </c>
       <c r="D2" t="n">
-        <v>87830.17999999999</v>
+        <v>24024745</v>
       </c>
       <c r="E2" t="n">
-        <v>24024745</v>
+        <v>89279.00999999999</v>
       </c>
       <c r="F2" t="n">
-        <v>89279.00999999999</v>
-      </c>
-      <c r="G2" t="n">
         <v>15590.36</v>
       </c>
     </row>
@@ -488,18 +480,15 @@
         <v>2711</v>
       </c>
       <c r="C3" t="n">
-        <v>42965.26</v>
+        <v>27318</v>
       </c>
       <c r="D3" t="n">
-        <v>27318</v>
+        <v>10090749.62</v>
       </c>
       <c r="E3" t="n">
-        <v>10090749.62</v>
+        <v>28064.25</v>
       </c>
       <c r="F3" t="n">
-        <v>28064.25</v>
-      </c>
-      <c r="G3" t="n">
         <v>3722.15</v>
       </c>
     </row>
@@ -513,18 +502,15 @@
         <v>2279</v>
       </c>
       <c r="C4" t="n">
-        <v>42558.22</v>
+        <v>23919.95</v>
       </c>
       <c r="D4" t="n">
-        <v>23919.95</v>
+        <v>8208742.56</v>
       </c>
       <c r="E4" t="n">
-        <v>8208742.56</v>
+        <v>24601.52</v>
       </c>
       <c r="F4" t="n">
-        <v>24601.52</v>
-      </c>
-      <c r="G4" t="n">
         <v>3601.91</v>
       </c>
     </row>
@@ -538,18 +524,15 @@
         <v>6531</v>
       </c>
       <c r="C5" t="n">
-        <v>253819.63</v>
+        <v>139068.13</v>
       </c>
       <c r="D5" t="n">
-        <v>139068.13</v>
+        <v>42324237.18</v>
       </c>
       <c r="E5" t="n">
-        <v>42324237.18</v>
+        <v>141944.78</v>
       </c>
       <c r="F5" t="n">
-        <v>141944.78</v>
-      </c>
-      <c r="G5" t="n">
         <v>6480.51</v>
       </c>
     </row>

</xml_diff>